<commit_message>
updated w local (fork)
</commit_message>
<xml_diff>
--- a/Inst/extdata/factor_recode.xlsx
+++ b/Inst/extdata/factor_recode.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B118"/>
+  <dimension ref="A1:B160"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -1540,6 +1540,426 @@
       <c r="B118" t="inlineStr">
         <is>
           <t>Stopped by transmitter: Sensor Failed 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2">
+        <v>45281.73700767361</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Started by xDrip</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2">
+        <v>45281.74649844908</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>ananas+blueberries 30min ago</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2">
+        <v>45281.85054452546</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>rice+p.chops+brussel sprouts+bonbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2">
+        <v>45282.32154039352</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>rice+p.chops+brussel sprouts+bonbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2">
+        <v>45282.58980795139</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>rice+beans+veal → rice+beans+veal+chocolate</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2">
+        <v>45282.78280341435</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>peanuts150+nuts100+honey60 → peanuts150+nutz100+honey60-ate 80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2">
+        <v>45283.36835873843</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>coffee w. oil</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2">
+        <v>45283.47350318287</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>bubble tea</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2">
+        <v>45283.59363346065</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>felt hypogl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2">
+        <v>45283.60949615741</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>buns+veal+paté+sweets</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2">
+        <v>45284.40338784723</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>almond150 → almond100</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2">
+        <v>45284.53489182871</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>pulyka+krumpli+bejgli</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2">
+        <v>45284.84882932871</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>turkey+bejgli</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2">
+        <v>45285.44408671296</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Snickers bar 50gr</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2">
+        <v>45285.51317083334</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>hungry, medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2">
+        <v>45285.55297765046</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>pogácsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2">
+        <v>45285.75634616899</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>aspique → aspique+jam+bonbon+stuff</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2">
+        <v>45286.38469148148</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>oat bran60+peas+turkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2">
+        <v>45286.53797002314</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>hungry-medium → potato</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2">
+        <v>45286.54368923611</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>cake decorating (not no caloric :)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2">
+        <v>45286.67021670139</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>white chocolate mud cake</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2">
+        <v>45287.36856089121</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>white chocolate mud cake</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2">
+        <v>45287.55955076389</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>coffee w milk100</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2">
+        <v>45287.57462168981</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>hamburger 30dkg meat</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2">
+        <v>45288.35324186343</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>cake kikelet (sugar free)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2">
+        <v>45288.5761821412</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>coffee w milk</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2">
+        <v>45288.59560060185</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2">
+        <v>45288.63096240741</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>futás vége</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2">
+        <v>45288.67249704861</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>dinner (turkey bread pate kikelet cake)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2">
+        <v>45288.8670471875</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>grapefruit → ananas</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>45289.22719980324</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>white chocolate mud cake</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2">
+        <v>45289.53480840278</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>white chocolate mud cake</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2">
+        <v>45289.71430209491</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>bread+eggs+tuna → +grapefruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2">
+        <v>45289.84719590278</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ananas</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2">
+        <v>45290.34066017361</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>eggs+bun</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2">
+        <v>45290.40833333333</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2">
+        <v>45290.52581949074</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Nagy kakas burger → +bubble tea</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2">
+        <v>45290.6182359375</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2">
+        <v>45290.80296393519</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>potatoes cake citrus</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2">
+        <v>45291.3265975</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>coffee</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2">
+        <v>45291.46628324074</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>citrus</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2">
+        <v>45291.51790640046</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>sushi</t>
         </is>
       </c>
     </row>
@@ -1773,9 +2193,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC04FD33-E8B5-40AA-B747-36F39B2FC3EF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB50F32B-D728-4CFE-98BC-3DFAE29E9722}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{970515D1-4B84-45D4-BE3A-205923B94B41}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF007963-E7EF-43EE-9F03-41D182B21AF3}"/>
 </file>
</xml_diff>